<commit_message>
docs: added README and updated project report.
</commit_message>
<xml_diff>
--- a/Documentation/project_management/gantt_chart.xlsx
+++ b/Documentation/project_management/gantt_chart.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\OJ\Proton Drive\oliverjabmyers\My files\uni\diss\project_management\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\prog\diss\Screenwriting-Project-Dissertation\Documentation\project_management\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5B473B4-9B54-4805-8C9A-3628831A8E2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63D66D13-2864-4692-8E10-D0D96FE76AB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -187,9 +187,6 @@
     <t>Project Skeleton</t>
   </si>
   <si>
-    <t>Testing</t>
-  </si>
-  <si>
     <t>Report</t>
   </si>
   <si>
@@ -199,13 +196,16 @@
     <t>Scrivener Research</t>
   </si>
   <si>
-    <t>Increment #1</t>
+    <t>Increment #1 (Model Layer)</t>
   </si>
   <si>
-    <t>Increment #2</t>
+    <t>Increment #2 (ViewModel + OSF)</t>
   </si>
   <si>
-    <t>Increment #3</t>
+    <t>Increment #3 (ScriptEditor + Scene Navigator)</t>
+  </si>
+  <si>
+    <t>Increment #4 (Pdf Export + Bug Fixes)</t>
   </si>
 </sst>
 </file>
@@ -921,6 +921,9 @@
     <xf numFmtId="0" fontId="0" fillId="14" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="166" fontId="0" fillId="6" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
@@ -935,9 +938,6 @@
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1519,47 +1519,47 @@
       <c r="F1" s="76"/>
       <c r="H1" s="2"/>
       <c r="I1" s="8"/>
-      <c r="J1" s="96" t="str">
+      <c r="J1" s="91" t="str">
         <f>HYPERLINK("https://vertex42.link/HowToMakeAGanttChart","► Watch How to Make a Gantt Chart in Excel")</f>
         <v>► Watch How to Make a Gantt Chart in Excel</v>
       </c>
-      <c r="K1" s="96"/>
-      <c r="L1" s="96"/>
-      <c r="M1" s="96"/>
-      <c r="N1" s="96"/>
-      <c r="O1" s="96"/>
-      <c r="P1" s="96"/>
-      <c r="Q1" s="96"/>
-      <c r="R1" s="96"/>
-      <c r="S1" s="96"/>
-      <c r="T1" s="96"/>
-      <c r="U1" s="96"/>
-      <c r="V1" s="96"/>
-      <c r="W1" s="96"/>
-      <c r="X1" s="96"/>
-      <c r="Y1" s="96"/>
-      <c r="Z1" s="96"/>
-      <c r="AA1" s="96"/>
+      <c r="K1" s="91"/>
+      <c r="L1" s="91"/>
+      <c r="M1" s="91"/>
+      <c r="N1" s="91"/>
+      <c r="O1" s="91"/>
+      <c r="P1" s="91"/>
+      <c r="Q1" s="91"/>
+      <c r="R1" s="91"/>
+      <c r="S1" s="91"/>
+      <c r="T1" s="91"/>
+      <c r="U1" s="91"/>
+      <c r="V1" s="91"/>
+      <c r="W1" s="91"/>
+      <c r="X1" s="91"/>
+      <c r="Y1" s="91"/>
+      <c r="Z1" s="91"/>
+      <c r="AA1" s="91"/>
     </row>
     <row r="2" spans="1:120" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B2" s="9"/>
       <c r="D2" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="E2" s="94">
+      <c r="E2" s="95">
         <v>46041</v>
       </c>
-      <c r="F2" s="95"/>
+      <c r="F2" s="96"/>
     </row>
     <row r="3" spans="1:120" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B3" s="9"/>
       <c r="D3" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="E3" s="94">
-        <v>46065</v>
-      </c>
-      <c r="F3" s="95"/>
+      <c r="E3" s="95">
+        <v>46140</v>
+      </c>
+      <c r="F3" s="96"/>
     </row>
     <row r="4" spans="1:120" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D4" s="6" t="s">
@@ -1568,166 +1568,166 @@
       <c r="E4" s="7">
         <v>1</v>
       </c>
-      <c r="I4" s="91">
+      <c r="I4" s="92">
         <f>I5</f>
         <v>46041</v>
       </c>
-      <c r="J4" s="92"/>
-      <c r="K4" s="92"/>
-      <c r="L4" s="92"/>
-      <c r="M4" s="92"/>
-      <c r="N4" s="92"/>
-      <c r="O4" s="93"/>
-      <c r="P4" s="91">
+      <c r="J4" s="93"/>
+      <c r="K4" s="93"/>
+      <c r="L4" s="93"/>
+      <c r="M4" s="93"/>
+      <c r="N4" s="93"/>
+      <c r="O4" s="94"/>
+      <c r="P4" s="92">
         <f>P5</f>
         <v>46048</v>
       </c>
-      <c r="Q4" s="92"/>
-      <c r="R4" s="92"/>
-      <c r="S4" s="92"/>
-      <c r="T4" s="92"/>
-      <c r="U4" s="92"/>
-      <c r="V4" s="93"/>
-      <c r="W4" s="91">
+      <c r="Q4" s="93"/>
+      <c r="R4" s="93"/>
+      <c r="S4" s="93"/>
+      <c r="T4" s="93"/>
+      <c r="U4" s="93"/>
+      <c r="V4" s="94"/>
+      <c r="W4" s="92">
         <f>W5</f>
         <v>46055</v>
       </c>
-      <c r="X4" s="92"/>
-      <c r="Y4" s="92"/>
-      <c r="Z4" s="92"/>
-      <c r="AA4" s="92"/>
-      <c r="AB4" s="92"/>
-      <c r="AC4" s="93"/>
-      <c r="AD4" s="91">
+      <c r="X4" s="93"/>
+      <c r="Y4" s="93"/>
+      <c r="Z4" s="93"/>
+      <c r="AA4" s="93"/>
+      <c r="AB4" s="93"/>
+      <c r="AC4" s="94"/>
+      <c r="AD4" s="92">
         <f>AD5</f>
         <v>46062</v>
       </c>
-      <c r="AE4" s="92"/>
-      <c r="AF4" s="92"/>
-      <c r="AG4" s="92"/>
-      <c r="AH4" s="92"/>
-      <c r="AI4" s="92"/>
-      <c r="AJ4" s="93"/>
-      <c r="AK4" s="91">
+      <c r="AE4" s="93"/>
+      <c r="AF4" s="93"/>
+      <c r="AG4" s="93"/>
+      <c r="AH4" s="93"/>
+      <c r="AI4" s="93"/>
+      <c r="AJ4" s="94"/>
+      <c r="AK4" s="92">
         <f>AK5</f>
         <v>46069</v>
       </c>
-      <c r="AL4" s="92"/>
-      <c r="AM4" s="92"/>
-      <c r="AN4" s="92"/>
-      <c r="AO4" s="92"/>
-      <c r="AP4" s="92"/>
-      <c r="AQ4" s="93"/>
-      <c r="AR4" s="91">
+      <c r="AL4" s="93"/>
+      <c r="AM4" s="93"/>
+      <c r="AN4" s="93"/>
+      <c r="AO4" s="93"/>
+      <c r="AP4" s="93"/>
+      <c r="AQ4" s="94"/>
+      <c r="AR4" s="92">
         <f>AR5</f>
         <v>46076</v>
       </c>
-      <c r="AS4" s="92"/>
-      <c r="AT4" s="92"/>
-      <c r="AU4" s="92"/>
-      <c r="AV4" s="92"/>
-      <c r="AW4" s="92"/>
-      <c r="AX4" s="93"/>
-      <c r="AY4" s="91">
+      <c r="AS4" s="93"/>
+      <c r="AT4" s="93"/>
+      <c r="AU4" s="93"/>
+      <c r="AV4" s="93"/>
+      <c r="AW4" s="93"/>
+      <c r="AX4" s="94"/>
+      <c r="AY4" s="92">
         <f>AY5</f>
         <v>46083</v>
       </c>
-      <c r="AZ4" s="92"/>
-      <c r="BA4" s="92"/>
-      <c r="BB4" s="92"/>
-      <c r="BC4" s="92"/>
-      <c r="BD4" s="92"/>
-      <c r="BE4" s="93"/>
-      <c r="BF4" s="91">
+      <c r="AZ4" s="93"/>
+      <c r="BA4" s="93"/>
+      <c r="BB4" s="93"/>
+      <c r="BC4" s="93"/>
+      <c r="BD4" s="93"/>
+      <c r="BE4" s="94"/>
+      <c r="BF4" s="92">
         <f>BF5</f>
         <v>46090</v>
       </c>
-      <c r="BG4" s="92"/>
-      <c r="BH4" s="92"/>
-      <c r="BI4" s="92"/>
-      <c r="BJ4" s="92"/>
-      <c r="BK4" s="92"/>
-      <c r="BL4" s="93"/>
-      <c r="BM4" s="91">
+      <c r="BG4" s="93"/>
+      <c r="BH4" s="93"/>
+      <c r="BI4" s="93"/>
+      <c r="BJ4" s="93"/>
+      <c r="BK4" s="93"/>
+      <c r="BL4" s="94"/>
+      <c r="BM4" s="92">
         <f>BM5</f>
         <v>46097</v>
       </c>
-      <c r="BN4" s="92"/>
-      <c r="BO4" s="92"/>
-      <c r="BP4" s="92"/>
-      <c r="BQ4" s="92"/>
-      <c r="BR4" s="92"/>
-      <c r="BS4" s="93"/>
-      <c r="BT4" s="91">
+      <c r="BN4" s="93"/>
+      <c r="BO4" s="93"/>
+      <c r="BP4" s="93"/>
+      <c r="BQ4" s="93"/>
+      <c r="BR4" s="93"/>
+      <c r="BS4" s="94"/>
+      <c r="BT4" s="92">
         <f>BT5</f>
         <v>46104</v>
       </c>
-      <c r="BU4" s="92"/>
-      <c r="BV4" s="92"/>
-      <c r="BW4" s="92"/>
-      <c r="BX4" s="92"/>
-      <c r="BY4" s="92"/>
-      <c r="BZ4" s="93"/>
-      <c r="CA4" s="91">
+      <c r="BU4" s="93"/>
+      <c r="BV4" s="93"/>
+      <c r="BW4" s="93"/>
+      <c r="BX4" s="93"/>
+      <c r="BY4" s="93"/>
+      <c r="BZ4" s="94"/>
+      <c r="CA4" s="92">
         <f>CA5</f>
         <v>46111</v>
       </c>
-      <c r="CB4" s="92"/>
-      <c r="CC4" s="92"/>
-      <c r="CD4" s="92"/>
-      <c r="CE4" s="92"/>
-      <c r="CF4" s="92"/>
-      <c r="CG4" s="93"/>
-      <c r="CH4" s="91">
+      <c r="CB4" s="93"/>
+      <c r="CC4" s="93"/>
+      <c r="CD4" s="93"/>
+      <c r="CE4" s="93"/>
+      <c r="CF4" s="93"/>
+      <c r="CG4" s="94"/>
+      <c r="CH4" s="92">
         <f t="shared" ref="CH4" si="0">CH5</f>
         <v>46118</v>
       </c>
-      <c r="CI4" s="92"/>
-      <c r="CJ4" s="92"/>
-      <c r="CK4" s="92"/>
-      <c r="CL4" s="92"/>
-      <c r="CM4" s="92"/>
-      <c r="CN4" s="93"/>
-      <c r="CO4" s="91">
+      <c r="CI4" s="93"/>
+      <c r="CJ4" s="93"/>
+      <c r="CK4" s="93"/>
+      <c r="CL4" s="93"/>
+      <c r="CM4" s="93"/>
+      <c r="CN4" s="94"/>
+      <c r="CO4" s="92">
         <f t="shared" ref="CO4" si="1">CO5</f>
         <v>46125</v>
       </c>
-      <c r="CP4" s="92"/>
-      <c r="CQ4" s="92"/>
-      <c r="CR4" s="92"/>
-      <c r="CS4" s="92"/>
-      <c r="CT4" s="92"/>
-      <c r="CU4" s="93"/>
-      <c r="CV4" s="91">
+      <c r="CP4" s="93"/>
+      <c r="CQ4" s="93"/>
+      <c r="CR4" s="93"/>
+      <c r="CS4" s="93"/>
+      <c r="CT4" s="93"/>
+      <c r="CU4" s="94"/>
+      <c r="CV4" s="92">
         <f t="shared" ref="CV4" si="2">CV5</f>
         <v>46132</v>
       </c>
-      <c r="CW4" s="92"/>
-      <c r="CX4" s="92"/>
-      <c r="CY4" s="92"/>
-      <c r="CZ4" s="92"/>
-      <c r="DA4" s="92"/>
-      <c r="DB4" s="93"/>
-      <c r="DC4" s="91">
+      <c r="CW4" s="93"/>
+      <c r="CX4" s="93"/>
+      <c r="CY4" s="93"/>
+      <c r="CZ4" s="93"/>
+      <c r="DA4" s="93"/>
+      <c r="DB4" s="94"/>
+      <c r="DC4" s="92">
         <f t="shared" ref="DC4" si="3">DC5</f>
         <v>46139</v>
       </c>
-      <c r="DD4" s="92"/>
-      <c r="DE4" s="92"/>
-      <c r="DF4" s="92"/>
-      <c r="DG4" s="92"/>
-      <c r="DH4" s="92"/>
-      <c r="DI4" s="93"/>
-      <c r="DJ4" s="91">
+      <c r="DD4" s="93"/>
+      <c r="DE4" s="93"/>
+      <c r="DF4" s="93"/>
+      <c r="DG4" s="93"/>
+      <c r="DH4" s="93"/>
+      <c r="DI4" s="94"/>
+      <c r="DJ4" s="92">
         <f t="shared" ref="DJ4" si="4">DJ5</f>
         <v>46146</v>
       </c>
-      <c r="DK4" s="92"/>
-      <c r="DL4" s="92"/>
-      <c r="DM4" s="92"/>
-      <c r="DN4" s="92"/>
-      <c r="DO4" s="92"/>
-      <c r="DP4" s="93"/>
+      <c r="DK4" s="93"/>
+      <c r="DL4" s="93"/>
+      <c r="DM4" s="93"/>
+      <c r="DN4" s="93"/>
+      <c r="DO4" s="93"/>
+      <c r="DP4" s="94"/>
     </row>
     <row r="5" spans="1:120" x14ac:dyDescent="0.3">
       <c r="A5" s="6"/>
@@ -3569,7 +3569,7 @@
     <row r="14" spans="1:120" s="3" customFormat="1" ht="21.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A14" s="19"/>
       <c r="B14" s="31" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C14" s="32"/>
       <c r="D14" s="33">
@@ -3706,7 +3706,7 @@
       </c>
       <c r="C15" s="32"/>
       <c r="D15" s="33">
-        <v>0.3</v>
+        <v>1</v>
       </c>
       <c r="E15" s="34">
         <v>46051</v>
@@ -3839,7 +3839,7 @@
       </c>
       <c r="C16" s="32"/>
       <c r="D16" s="33">
-        <v>0.3</v>
+        <v>1</v>
       </c>
       <c r="E16" s="34">
         <v>46054</v>
@@ -3972,7 +3972,7 @@
       </c>
       <c r="C17" s="32"/>
       <c r="D17" s="33">
-        <v>0.7</v>
+        <v>1</v>
       </c>
       <c r="E17" s="34">
         <v>46059</v>
@@ -4101,11 +4101,11 @@
     <row r="18" spans="1:120" s="3" customFormat="1" ht="21.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A18" s="19"/>
       <c r="B18" s="31" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C18" s="32"/>
       <c r="D18" s="33">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="E18" s="34">
         <v>46060</v>
@@ -4365,7 +4365,7 @@
       </c>
       <c r="C20" s="42"/>
       <c r="D20" s="43">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E20" s="44">
         <v>46067</v>
@@ -4494,11 +4494,11 @@
     <row r="21" spans="1:120" s="3" customFormat="1" ht="21.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A21" s="19"/>
       <c r="B21" s="41" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C21" s="42"/>
       <c r="D21" s="43">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E21" s="44">
         <v>46067</v>
@@ -4627,11 +4627,11 @@
     <row r="22" spans="1:120" s="3" customFormat="1" ht="21.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A22" s="19"/>
       <c r="B22" s="41" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C22" s="42"/>
       <c r="D22" s="43">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E22" s="44">
         <v>46067</v>
@@ -4760,11 +4760,11 @@
     <row r="23" spans="1:120" s="3" customFormat="1" ht="21.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A23" s="19"/>
       <c r="B23" s="41" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C23" s="42"/>
       <c r="D23" s="43">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E23" s="44">
         <v>46067</v>
@@ -4893,11 +4893,11 @@
     <row r="24" spans="1:120" s="3" customFormat="1" ht="21.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A24" s="19"/>
       <c r="B24" s="41" t="s">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="C24" s="42"/>
       <c r="D24" s="43">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E24" s="44">
         <v>46067</v>
@@ -5153,20 +5153,22 @@
     <row r="26" spans="1:120" s="3" customFormat="1" ht="21.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A26" s="19"/>
       <c r="B26" s="51" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C26" s="52"/>
-      <c r="D26" s="53"/>
+      <c r="D26" s="53">
+        <v>0.9</v>
+      </c>
       <c r="E26" s="54">
-        <v>43481</v>
+        <v>46132</v>
       </c>
       <c r="F26" s="55">
-        <v>43486</v>
+        <v>46143</v>
       </c>
       <c r="G26" s="25"/>
       <c r="H26" s="25">
         <f t="shared" si="62"/>
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="I26" s="62"/>
       <c r="J26" s="62"/>
@@ -7758,17 +7760,6 @@
     </row>
   </sheetData>
   <mergeCells count="19">
-    <mergeCell ref="J1:AA1"/>
-    <mergeCell ref="AK4:AQ4"/>
-    <mergeCell ref="AR4:AX4"/>
-    <mergeCell ref="AY4:BE4"/>
-    <mergeCell ref="BF4:BL4"/>
-    <mergeCell ref="E2:F2"/>
-    <mergeCell ref="I4:O4"/>
-    <mergeCell ref="P4:V4"/>
-    <mergeCell ref="W4:AC4"/>
-    <mergeCell ref="AD4:AJ4"/>
-    <mergeCell ref="E3:F3"/>
     <mergeCell ref="CV4:DB4"/>
     <mergeCell ref="DC4:DI4"/>
     <mergeCell ref="DJ4:DP4"/>
@@ -7777,6 +7768,17 @@
     <mergeCell ref="CA4:CG4"/>
     <mergeCell ref="CH4:CN4"/>
     <mergeCell ref="CO4:CU4"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="I4:O4"/>
+    <mergeCell ref="P4:V4"/>
+    <mergeCell ref="W4:AC4"/>
+    <mergeCell ref="AD4:AJ4"/>
+    <mergeCell ref="E3:F3"/>
+    <mergeCell ref="J1:AA1"/>
+    <mergeCell ref="AK4:AQ4"/>
+    <mergeCell ref="AR4:AX4"/>
+    <mergeCell ref="AY4:BE4"/>
+    <mergeCell ref="BF4:BL4"/>
   </mergeCells>
   <conditionalFormatting sqref="D7:D46">
     <cfRule type="dataBar" priority="12">

</xml_diff>